<commit_message>
docs: switch due-diligence dev scenario to solo AI-first developer (S1)
Recompute roadmap, financial model, executive summary and risk register
around the S1 (1 AI-first developer) scenario instead of S2: lower team
Opex ($5.5K/mo vs $9K), longer/less risk-tolerant timeline to MVP
(realistic 5.1mo / pessimistic 9.3mo vs 3.2/5.8mo for S2), earlier
break-even by MAU (~37-46K vs ~55-73K) due to lower fixed costs, and an
explicit bus-factor-1 risk entry with mitigation (external audit before
payments launch, decisions documented as they're made).
</commit_message>
<xml_diff>
--- a/docs/due-diligence/syntx/models/financial-model.xlsx
+++ b/docs/due-diligence/syntx/models/financial-model.xlsx
@@ -2256,15 +2256,15 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Team cost (S2: 2 разработчика + fractional PM/design)</t>
+          <t>Team cost (S1: 1 AI-first разработчик + fractional legal/design)</t>
         </is>
       </c>
       <c r="B43" s="4" t="n">
-        <v>9000</v>
+        <v>5500</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>USD/мес, см. 08</t>
+          <t>USD/мес — $220/день x 20 дней (см. 08) + ~$1,100 на подрядчиков</t>
         </is>
       </c>
     </row>

</xml_diff>